<commit_message>
Fix XLSForm converter: all 16 sample scales pass pyxform validation
- parameter conditions in visible_when skipped (not runtime fields)
- scoring calculate fields moved to top level (ODK rejects groups with only calculates)
- calculate XPath filters to items present in flattened form (fixes variant scales like EWS/PAS)
- blank-label section/inst notes suppressed (pyxform requires note label)
- Update xlsform_samples/ with pyxform-validated outputs

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/xlsform_samples/ACE.xlsx
+++ b/tools/xlsform_samples/ACE.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1238,28 +1238,28 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ACE_scoring</t>
+          <t>ACE_commitment</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Computed Scores</t>
+          <t>commitment (mean_coded)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>field-list</t>
-        </is>
-      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>((${ace1} + ${ace2} + ${ace3} + ${ace4} + ${ace5} + ${ace6}) div 6) * 6.25</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
@@ -1273,12 +1273,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ACE_commitment</t>
+          <t>ACE_informed_choice</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>commitment (mean_coded)</t>
+          <t>informed_choice (mean_coded)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1286,7 +1286,7 @@
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>((${ace1} + ${ace2} + ${ace3} + ${ace4} + ${ace5} + ${ace6}) div 6) * 6.25</t>
+          <t>((${ace7} + ${ace8} + ${ace9} + ${ace10} + ${ace11}) div 5) * 6.25</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
@@ -1303,12 +1303,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ACE_informed_choice</t>
+          <t>ACE_navigation</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>informed_choice (mean_coded)</t>
+          <t>navigation (mean_coded)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1316,7 +1316,7 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>((${ace7} + ${ace8} + ${ace9} + ${ace10} + ${ace11}) div 5) * 6.25</t>
+          <t>((${ace12} + ${ace13} + ${ace14} + ${ace15} + ${ace16}) div 5) * 6.25</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
@@ -1333,12 +1333,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ACE_navigation</t>
+          <t>ACE_ownership</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>navigation (mean_coded)</t>
+          <t>ownership (mean_coded)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1346,7 +1346,7 @@
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>((${ace12} + ${ace13} + ${ace14} + ${ace15} + ${ace16}) div 5) * 6.25</t>
+          <t>((${ace17} + ${ace18} + ${ace19} + ${ace20} + ${ace21}) div 5) * 6.25</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
@@ -1363,12 +1363,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ACE_ownership</t>
+          <t>ACE_ace_total</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ownership (mean_coded)</t>
+          <t>ace_total (sum_coded)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1376,7 +1376,7 @@
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>((${ace17} + ${ace18} + ${ace19} + ${ace20} + ${ace21}) div 5) * 6.25</t>
+          <t>${ACE_commitment} + ${ACE_informed_choice} + ${ACE_navigation} + ${ACE_ownership}</t>
         </is>
       </c>
       <c r="H27" t="inlineStr"/>
@@ -1384,58 +1384,6 @@
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>calculate</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>ACE_ace_total</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>ace_total (sum_coded)</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>${ACE_commitment} + ${ACE_informed_choice} + ${ACE_navigation} + ${ACE_ownership}</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>end group</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>ACE_scoring</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Set default_language='English (en)' in settings sheet; rebuild samples
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/xlsform_samples/ACE.xlsx
+++ b/tools/xlsform_samples/ACE.xlsx
@@ -1564,7 +1564,11 @@
           <t>20260618</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>English (en)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>